<commit_message>
Regenerate glove tracker workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BLuvBpaPW5Ciq6CtNVqHGy
</commit_message>
<xml_diff>
--- a/glove_tracker.xlsx
+++ b/glove_tracker.xlsx
@@ -975,11 +975,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="58389262"/>
-        <c:axId val="50225220"/>
+        <c:axId val="94029016"/>
+        <c:axId val="35119304"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="58389262"/>
+        <c:axId val="94029016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1011,7 +1011,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50225220"/>
+        <c:crossAx val="35119304"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1019,7 +1019,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50225220"/>
+        <c:axId val="35119304"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1095,7 +1095,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58389262"/>
+        <c:crossAx val="94029016"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>